<commit_message>
Add charts and advanced sales analysis
</commit_message>
<xml_diff>
--- a/output/report.xlsx
+++ b/output/report.xlsx
@@ -7,7 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales by Category" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profit by Category" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Sub-Categories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Sales" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,49 +442,723 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>836154.0330000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>741999.7953</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>719047.032</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Profit</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>145454.9481</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>122490.8008</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Furniture</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>18451.2728</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Phones</t>
+        </is>
+      </c>
       <c r="B2" t="n">
-        <v>741999.7953</v>
-      </c>
-      <c r="C2" t="n">
-        <v>18451.2728</v>
+        <v>330007.054</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Office Supplies</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Chairs</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>719047.032</v>
-      </c>
-      <c r="C3" t="n">
-        <v>122490.8008</v>
+        <v>328449.103</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Technology</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Storage</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>836154.0330000001</v>
-      </c>
-      <c r="C4" t="n">
-        <v>145454.9481</v>
+        <v>223843.608</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tables</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>206965.532</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Binders</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>203412.733</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Machines</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>189238.631</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>167380.318</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Copiers</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>149528.03</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bookcases</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>114879.9963</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>107532.161</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>YearMonth</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2014-01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>14236.895</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2014-02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4519.892</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2014-03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>55691.009</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2014-04</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>28295.345</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2014-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>23648.287</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2014-06</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>34595.1276</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2014-07</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>33946.393</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2014-08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>27909.4685</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2014-09</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>81777.3508</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2014-10</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>31453.393</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2014-11</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>78628.7167</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2014-12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>69545.6205</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2015-01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>18174.0756</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2015-02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>11951.411</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2015-03</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>38726.252</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2015-04</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>34195.2085</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2015-05</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>30131.6865</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2015-06</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>24797.292</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2015-07</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>28765.325</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2015-08</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>36898.3322</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2015-09</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>64595.918</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2015-10</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>31404.9235</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2015-11</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>75972.5635</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2015-12</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>74919.5212</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2016-01</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>18542.491</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2016-02</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>22978.815</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2016-03</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>51715.875</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2016-04</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>38750.039</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2016-05</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>56987.728</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2016-06</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>40344.534</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2016-07</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>39261.963</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2016-08</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>31115.3743</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2016-09</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>73410.0249</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2016-10</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>59687.745</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2016-11</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>79411.96580000001</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2016-12</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>96999.04300000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2017-01</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>43971.374</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2017-02</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>20301.1334</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2017-03</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>58872.3528</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2017-04</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>36521.5361</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2017-05</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>44261.1102</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2017-06</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>52981.7257</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2017-07</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>45264.416</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2017-08</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>63120.888</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2017-09</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>87866.652</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2017-10</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>77776.9232</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2017-11</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>118447.825</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2017-12</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>83829.31879999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>